<commit_message>
Load the cached catalog before the old bootstrap fallback on startup
load_initial() tried the bootstrap paths (products.xlsx, then the very
first sample CSV checked into the repo root) before ever checking the
cache file - since the sample CSV loads successfully, it always won on
a fresh start, silently skipping the more current cached catalog (the
result of the last real Zoho pull or manual upload) sitting right next
to it. This matters more now that the daily Zoho pull is off: a fresh
deploy/restart with no persistent disk needs its bootstrap data to
actually be the most recent snapshot, not permanently stuck on old
sample data. Cache is now checked first; the old paths are the true
last resort. Also updates the committed cache snapshot itself to
today's real 73-product pull so this fix ships with current data, not
the stale 82-row one.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/.cache/products_catalog.xlsx
+++ b/.cache/products_catalog.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" r:id="rId1" sheetId="1"/>
+    <sheet name="Hampers" r:id="rId2" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
   <si>
     <t>Better for you Options</t>
   </si>
@@ -297,6 +298,156 @@
   </si>
   <si>
     <t>Maaza</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>length</t>
+  </si>
+  <si>
+    <t>breadth</t>
+  </si>
+  <si>
+    <t>height</t>
+  </si>
+  <si>
+    <t>LED tealight candle</t>
+  </si>
+  <si>
+    <t>Besan Laddoo Cookies 100g</t>
+  </si>
+  <si>
+    <t>Inside item</t>
+  </si>
+  <si>
+    <t>Achari Aam Crackers 100g</t>
+  </si>
+  <si>
+    <t>Rava Laddoo Cookies 100g</t>
+  </si>
+  <si>
+    <t>Cheesy Chand Crunch 70g</t>
+  </si>
+  <si>
+    <t>Baked Mathri 75g</t>
+  </si>
+  <si>
+    <t>Pack of 2 (3x1x1.7 inch) chocolate</t>
+  </si>
+  <si>
+    <t>Chocolate (pack of 4)</t>
+  </si>
+  <si>
+    <t>Ajwain Cookies</t>
+  </si>
+  <si>
+    <t>Truffle (pack of 9)</t>
+  </si>
+  <si>
+    <t>Cinnamon hot chocolate</t>
+  </si>
+  <si>
+    <t>Chocolate (2) + tea light candle (2)</t>
+  </si>
+  <si>
+    <t>soy wax tea light (2)</t>
+  </si>
+  <si>
+    <t>Farmley mixed nuts 21g</t>
+  </si>
+  <si>
+    <t>Tealight candle (pack of 2)</t>
+  </si>
+  <si>
+    <t>Elephants tea light holder</t>
+  </si>
+  <si>
+    <t>Tote Bag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MDF Tray 10x6 - 270/- </t>
+  </si>
+  <si>
+    <t>Hamper box</t>
+  </si>
+  <si>
+    <t>Small lamp</t>
+  </si>
+  <si>
+    <t>Craft Lantern</t>
+  </si>
+  <si>
+    <t>Tealight pack of 4</t>
+  </si>
+  <si>
+    <t>11 x 4.5 x 2.5 inch box - bougenvilla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13.5 x 7 x 3.5 inch box - blue </t>
+  </si>
+  <si>
+    <t>10 x 10 x 3 w cavity - Jaipur palace</t>
+  </si>
+  <si>
+    <t>10 x 10 x 3 w/o cavity - Jaipur palace</t>
+  </si>
+  <si>
+    <t>10 x 10 x 3 - 9 inch</t>
+  </si>
+  <si>
+    <t>Greeting Card</t>
+  </si>
+  <si>
+    <t>Lotus Bowl</t>
+  </si>
+  <si>
+    <t>Chocolate Bar</t>
+  </si>
+  <si>
+    <t>Dry fruit 200g tin - almond</t>
+  </si>
+  <si>
+    <t>Brass Lamp</t>
+  </si>
+  <si>
+    <t>Phool incense cone</t>
+  </si>
+  <si>
+    <t>Dry fruit 200g tin - cashew</t>
+  </si>
+  <si>
+    <t>Dry fruit 200g tin - raisin</t>
+  </si>
+  <si>
+    <t>Dry fruit 150g tin - nutty mix</t>
+  </si>
+  <si>
+    <t>Dry fruit 150g tin - almond</t>
+  </si>
+  <si>
+    <t>Dry fruit 200g tin - nutty mix</t>
+  </si>
+  <si>
+    <t>Dry fruit 100g tin - nutty mix</t>
+  </si>
+  <si>
+    <t>Besan small tin</t>
+  </si>
+  <si>
+    <t>Gingerbread cookies</t>
+  </si>
+  <si>
+    <t>Guntur Piri Piri</t>
+  </si>
+  <si>
+    <t>Besan hexagon</t>
+  </si>
+  <si>
+    <t>Rava Hexagon</t>
+  </si>
+  <si>
+    <t>Achari Hexagon</t>
   </si>
 </sst>
 </file>
@@ -309,29 +460,34 @@
   <fonts count="6">
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Roboto"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <color theme="1"/>
       <name val="Roboto"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Roboto"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Roboto"/>
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
       <name val="Roboto"/>
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Roboto"/>
     </font>
   </fonts>
@@ -415,60 +571,63 @@
       <alignment vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0">
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="2" numFmtId="0" xfId="0">
+    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0">
+    <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="164" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="2" fillId="0" fontId="0" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="164" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0">
+    <xf borderId="3" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="4" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0">
+    <xf borderId="3" fillId="0" fontId="0" numFmtId="164" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="164" xfId="0">
+    <xf borderId="4" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="164" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="1" numFmtId="164" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -487,6 +646,316 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="3C4F63"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="F4F6F6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="3498DB"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="2ECC71"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="F1C40F"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="E67622"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="EE4675"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="9B59B6"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="185C8A"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="3A62C8"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Roboto"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Roboto"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
   <dimension ref="A1:H83"/>
@@ -2788,4 +3257,320 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr defaultRowHeight="14.0" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="34.44"/>
+    <col min="2" max="2048" width="13.24"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11">
+        <v>5.0</v>
+      </c>
+      <c r="D11">
+        <v>5.0</v>
+      </c>
+      <c r="E11">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>110</v>
+      </c>
+      <c r="B12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B14" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B15" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>114</v>
+      </c>
+      <c r="B16" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>115</v>
+      </c>
+      <c r="B17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>116</v>
+      </c>
+      <c r="B18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C18">
+        <v>3.0</v>
+      </c>
+      <c r="D18">
+        <v>3.0</v>
+      </c>
+      <c r="E18">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>144</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>